<commit_message>
the expanse is done
</commit_message>
<xml_diff>
--- a/public/VASM Inputs.xlsx
+++ b/public/VASM Inputs.xlsx
@@ -8,20 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bharath/Documents/Innovative/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04452E02-9E9C-2946-BC93-36195623BE4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61CA840B-542C-8B49-A487-3724C5A34350}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="360" yWindow="1540" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SUMMARY" sheetId="2" r:id="rId1"/>
     <sheet name="REVENUE" sheetId="4" r:id="rId2"/>
     <sheet name="EXPENSES" sheetId="3" r:id="rId3"/>
     <sheet name="EXPENSES_01" sheetId="5" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="6" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">EXPENSES!$C$2:$M$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">EXPENSES_01!#REF!</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">REVENUE!$A$1:$AA$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">REVENUE!$A$1:$Y$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">SUMMARY!#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -45,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="148">
   <si>
     <t>CUSTOMER</t>
   </si>
@@ -296,9 +297,6 @@
     <t>DUE DAYS</t>
   </si>
   <si>
-    <t>BU HEAD ENTRY</t>
-  </si>
-  <si>
     <t>Auto pop up for Accounts</t>
   </si>
   <si>
@@ -426,10 +424,6 @@
   </si>
   <si>
     <t>FIRM</t>
-  </si>
-  <si>
-    <t>FROM VRP MASTER DATA 
-AND MANUAL ENTRY</t>
   </si>
   <si>
     <t>SL No</t>
@@ -579,7 +573,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -634,6 +628,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="20">
     <border>
@@ -908,7 +908,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1148,6 +1148,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1455,34 +1458,34 @@
         <v>3</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C1" s="13" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E1" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="F1" s="13" t="s">
         <v>111</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="G1" s="13" t="s">
         <v>112</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="H1" s="13" t="s">
         <v>113</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="I1" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="I1" s="13" t="s">
+      <c r="J1" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="J1" s="13" t="s">
+      <c r="K1" s="13" t="s">
         <v>116</v>
-      </c>
-      <c r="K1" s="13" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="19" x14ac:dyDescent="0.25">
@@ -1649,10 +1652,10 @@
         <v>61</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G12" s="11" t="s">
         <v>73</v>
@@ -1664,10 +1667,10 @@
         <v>64</v>
       </c>
       <c r="J12" s="11" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="K12" s="11" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="22" thickBot="1" x14ac:dyDescent="0.25">
@@ -1748,7 +1751,7 @@
         <v>3</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C1" s="13" t="s">
         <v>2</v>
@@ -1760,13 +1763,13 @@
         <v>0</v>
       </c>
       <c r="F1" s="13" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G1" s="14" t="s">
         <v>4</v>
       </c>
       <c r="H1" s="14" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I1" s="14" t="s">
         <v>11</v>
@@ -1790,7 +1793,7 @@
         <v>44</v>
       </c>
       <c r="P1" s="13" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="Q1" s="13" t="s">
         <v>43</v>
@@ -2382,7 +2385,7 @@
         <v>67</v>
       </c>
       <c r="P12" s="11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="Q12" s="11" t="s">
         <v>64</v>
@@ -2417,12 +2420,8 @@
       </c>
     </row>
     <row r="13" spans="1:27" ht="45" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C13" s="45" t="s">
-        <v>72</v>
-      </c>
-      <c r="K13" s="45" t="s">
-        <v>78</v>
-      </c>
+      <c r="C13" s="81"/>
+      <c r="K13" s="81"/>
       <c r="L13" s="45" t="s">
         <v>72</v>
       </c>
@@ -2430,7 +2429,7 @@
         <v>73</v>
       </c>
       <c r="P13" s="45" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="Q13" s="45" t="s">
         <v>72</v>
@@ -2446,7 +2445,7 @@
       <c r="O14" s="1"/>
       <c r="P14" s="1"/>
       <c r="W14" s="45" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="18" spans="6:9" x14ac:dyDescent="0.2">
@@ -2483,7 +2482,7 @@
       <c r="I24" s="1"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Y11" xr:uid="{B43AE799-94D2-4DA5-8971-DAD37CE6B6EE}"/>
+  <autoFilter ref="A1:Y14" xr:uid="{B43AE799-94D2-4DA5-8971-DAD37CE6B6EE}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -2511,7 +2510,7 @@
   <sheetData>
     <row r="1" spans="2:13" ht="55.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C1" s="78" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D1" s="79"/>
       <c r="E1" s="79"/>
@@ -2526,43 +2525,41 @@
     </row>
     <row r="2" spans="2:13" s="1" customFormat="1" ht="23" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C2" s="12" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E2" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="F2" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="G2" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="G2" s="14" t="s">
+      <c r="H2" s="13" t="s">
         <v>88</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="I2" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="J2" s="14" t="s">
         <v>89</v>
       </c>
-      <c r="I2" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="J2" s="14" t="s">
-        <v>90</v>
-      </c>
       <c r="K2" s="13" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="L2" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="M2" s="14" t="s">
         <v>92</v>
       </c>
-      <c r="M2" s="14" t="s">
-        <v>93</v>
-      </c>
     </row>
     <row r="3" spans="2:13" ht="19" x14ac:dyDescent="0.25">
-      <c r="B3" s="75" t="s">
-        <v>120</v>
-      </c>
+      <c r="B3" s="75"/>
       <c r="C3" s="55">
         <v>1</v>
       </c>
@@ -2732,7 +2729,7 @@
         <v>62</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G13" s="11" t="s">
         <v>61</v>
@@ -2759,7 +2756,7 @@
     <row r="15" spans="2:13" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="16" spans="2:13" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C16" s="78" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D16" s="79"/>
       <c r="E16" s="79"/>
@@ -2773,25 +2770,25 @@
     </row>
     <row r="17" spans="2:18" s="1" customFormat="1" ht="23" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C17" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="D17" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="E17" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="F17" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="G17" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="H17" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="D17" s="13" t="s">
-        <v>119</v>
-      </c>
-      <c r="E17" s="13" t="s">
-        <v>86</v>
-      </c>
-      <c r="F17" s="13" t="s">
+      <c r="I17" s="14" t="s">
         <v>96</v>
-      </c>
-      <c r="G17" s="13" t="s">
-        <v>124</v>
-      </c>
-      <c r="H17" s="13" t="s">
-        <v>123</v>
-      </c>
-      <c r="I17" s="14" t="s">
-        <v>97</v>
       </c>
       <c r="J17"/>
       <c r="K17"/>
@@ -2800,9 +2797,7 @@
       <c r="N17"/>
     </row>
     <row r="18" spans="2:18" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="75" t="s">
-        <v>120</v>
-      </c>
+      <c r="B18" s="75"/>
       <c r="C18" s="2">
         <v>1</v>
       </c>
@@ -2963,7 +2958,7 @@
         <v>62</v>
       </c>
       <c r="F28" s="11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G28" s="11" t="s">
         <v>61</v>
@@ -2986,7 +2981,7 @@
     <row r="31" spans="2:18" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="32" spans="2:18" ht="27" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C32" s="78" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D32" s="79"/>
       <c r="E32" s="79"/>
@@ -3008,58 +3003,56 @@
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="12" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D33" s="13" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E33" s="13" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F33" s="13" t="s">
         <v>4</v>
       </c>
       <c r="G33" s="14" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H33" s="13" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I33" s="14" t="s">
         <v>74</v>
       </c>
       <c r="J33" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="K33" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="L33" s="14" t="s">
         <v>101</v>
       </c>
-      <c r="K33" s="14" t="s">
-        <v>101</v>
-      </c>
-      <c r="L33" s="14" t="s">
+      <c r="M33" s="14" t="s">
         <v>102</v>
       </c>
-      <c r="M33" s="14" t="s">
+      <c r="N33" s="14" t="s">
         <v>103</v>
       </c>
-      <c r="N33" s="14" t="s">
+      <c r="O33" s="14" t="s">
         <v>104</v>
       </c>
-      <c r="O33" s="14" t="s">
+      <c r="P33" s="14" t="s">
         <v>105</v>
       </c>
-      <c r="P33" s="14" t="s">
+      <c r="Q33" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="R33" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="Q33" s="14" t="s">
-        <v>106</v>
-      </c>
-      <c r="R33" s="14" t="s">
-        <v>107</v>
-      </c>
     </row>
     <row r="34" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="75" t="s">
-        <v>120</v>
-      </c>
+      <c r="B34" s="75"/>
       <c r="C34" s="55">
         <v>1</v>
       </c>
@@ -3279,13 +3272,13 @@
         <v>62</v>
       </c>
       <c r="F44" s="11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G44" s="11" t="s">
         <v>61</v>
       </c>
       <c r="H44" s="11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I44" s="11" t="s">
         <v>61</v>
@@ -3315,7 +3308,7 @@
         <v>64</v>
       </c>
       <c r="R44" s="11" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="50" spans="4:4" x14ac:dyDescent="0.2">
@@ -3338,10 +3331,10 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E37E81B5-418A-45CE-B377-01D7348B71CD}">
-  <dimension ref="B1:L40"/>
+  <dimension ref="A1:L40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.33203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="14.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27" style="1" customWidth="1"/>
     <col min="4" max="4" width="30.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="24.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="26.5" customWidth="1"/>
@@ -3356,583 +3349,812 @@
     <col min="16" max="18" width="15.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:10" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="2:10" ht="23" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="57" t="s">
-        <v>121</v>
-      </c>
-      <c r="C2" s="57" t="s">
+    <row r="1" spans="1:9" ht="45" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="57" t="s">
         <v>119</v>
       </c>
-      <c r="D2" s="57" t="s">
+      <c r="B1" s="57" t="s">
+        <v>118</v>
+      </c>
+      <c r="C1" s="57" t="s">
+        <v>123</v>
+      </c>
+      <c r="D1" s="57" t="s">
+        <v>124</v>
+      </c>
+      <c r="E1" s="57" t="s">
+        <v>99</v>
+      </c>
+      <c r="F1" s="57" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="57" t="s">
+        <v>74</v>
+      </c>
+      <c r="H1" s="57" t="s">
+        <v>4</v>
+      </c>
+      <c r="I1" s="57" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+      <c r="A2" s="59">
+        <v>1</v>
+      </c>
+      <c r="B2" s="60"/>
+      <c r="C2" s="63" t="s">
+        <v>138</v>
+      </c>
+      <c r="D2" s="62"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
+      <c r="H2" s="61"/>
+      <c r="I2" s="64"/>
+    </row>
+    <row r="3" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+      <c r="A3" s="65">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2"/>
+      <c r="C3" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="D3" s="4"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="66"/>
+    </row>
+    <row r="4" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+      <c r="A4" s="65">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2"/>
+      <c r="C4" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="E2" s="57" t="s">
-        <v>126</v>
-      </c>
-      <c r="F2" s="57" t="s">
-        <v>100</v>
-      </c>
-      <c r="G2" s="57" t="s">
-        <v>4</v>
-      </c>
-      <c r="H2" s="57" t="s">
-        <v>74</v>
-      </c>
-      <c r="I2" s="57" t="s">
-        <v>4</v>
-      </c>
-      <c r="J2" s="57" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="2:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="B3" s="59">
-        <v>1</v>
-      </c>
-      <c r="C3" s="60"/>
-      <c r="D3" s="63" t="s">
-        <v>140</v>
-      </c>
-      <c r="E3" s="62"/>
-      <c r="F3" s="63"/>
-      <c r="G3" s="63"/>
-      <c r="H3" s="63"/>
-      <c r="I3" s="61"/>
-      <c r="J3" s="64"/>
-    </row>
-    <row r="4" spans="2:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="B4" s="65">
-        <v>2</v>
-      </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="E4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="5"/>
       <c r="F4" s="5"/>
       <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="66"/>
-    </row>
-    <row r="5" spans="2:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="B5" s="65">
-        <v>3</v>
-      </c>
-      <c r="C5" s="2"/>
-      <c r="D5" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="E5" s="4"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="66"/>
+    </row>
+    <row r="5" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+      <c r="A5" s="65">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="D5" s="4"/>
+      <c r="E5" s="5"/>
       <c r="F5" s="5"/>
       <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="3"/>
-      <c r="J5" s="66"/>
-    </row>
-    <row r="6" spans="2:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="B6" s="65">
-        <v>4</v>
-      </c>
-      <c r="C6" s="2"/>
-      <c r="D6" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="E6" s="4"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="66"/>
+    </row>
+    <row r="6" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+      <c r="A6" s="65">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2"/>
+      <c r="C6" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="D6" s="4"/>
+      <c r="E6" s="5"/>
       <c r="F6" s="5"/>
       <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="3"/>
-      <c r="J6" s="66"/>
-    </row>
-    <row r="7" spans="2:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="B7" s="65">
-        <v>5</v>
-      </c>
-      <c r="C7" s="2"/>
-      <c r="D7" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="E7" s="4"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="66"/>
+    </row>
+    <row r="7" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+      <c r="A7" s="65">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2"/>
+      <c r="C7" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="D7" s="4"/>
+      <c r="E7" s="5"/>
       <c r="F7" s="5"/>
       <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="3"/>
-      <c r="J7" s="66"/>
-    </row>
-    <row r="8" spans="2:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="B8" s="65">
-        <v>6</v>
-      </c>
-      <c r="C8" s="2"/>
-      <c r="D8" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="E8" s="4"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="66"/>
+    </row>
+    <row r="8" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+      <c r="A8" s="65">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2"/>
+      <c r="C8" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="D8" s="4"/>
+      <c r="E8" s="5"/>
       <c r="F8" s="5"/>
       <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="3"/>
-      <c r="J8" s="66"/>
-    </row>
-    <row r="9" spans="2:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="B9" s="65">
-        <v>7</v>
-      </c>
-      <c r="C9" s="2"/>
-      <c r="D9" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="E9" s="4"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="66"/>
+    </row>
+    <row r="9" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+      <c r="A9" s="65">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2"/>
+      <c r="C9" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="D9" s="4"/>
+      <c r="E9" s="5"/>
       <c r="F9" s="5"/>
       <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="66"/>
-    </row>
-    <row r="10" spans="2:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="B10" s="65">
-        <v>8</v>
-      </c>
-      <c r="C10" s="2"/>
-      <c r="D10" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="E10" s="4"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="66"/>
+    </row>
+    <row r="10" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+      <c r="A10" s="65">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2"/>
+      <c r="C10" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="D10" s="4"/>
+      <c r="E10" s="5"/>
       <c r="F10" s="5"/>
       <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="3"/>
-      <c r="J10" s="66"/>
-    </row>
-    <row r="11" spans="2:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="B11" s="65">
-        <v>9</v>
-      </c>
-      <c r="C11" s="2"/>
-      <c r="D11" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="E11" s="4"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="66"/>
+    </row>
+    <row r="11" spans="1:9" ht="19" x14ac:dyDescent="0.2">
+      <c r="A11" s="67">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3"/>
+      <c r="C11" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="D11" s="58"/>
+      <c r="E11" s="5"/>
       <c r="F11" s="5"/>
       <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="3"/>
-      <c r="J11" s="66"/>
-    </row>
-    <row r="12" spans="2:10" ht="19" x14ac:dyDescent="0.2">
-      <c r="B12" s="67">
-        <v>10</v>
-      </c>
-      <c r="C12" s="3"/>
-      <c r="D12" s="5" t="s">
-        <v>147</v>
-      </c>
-      <c r="E12" s="58"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="68"/>
+    </row>
+    <row r="12" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+      <c r="A12" s="65">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2"/>
+      <c r="C12" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="D12" s="4"/>
+      <c r="E12" s="5"/>
       <c r="F12" s="5"/>
       <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="3"/>
-      <c r="J12" s="68"/>
-    </row>
-    <row r="13" spans="2:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="B13" s="65">
-        <v>11</v>
-      </c>
-      <c r="C13" s="2"/>
-      <c r="D13" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="E13" s="4"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="66"/>
+    </row>
+    <row r="13" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+      <c r="A13" s="65">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2"/>
+      <c r="C13" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="D13" s="4"/>
+      <c r="E13" s="5"/>
       <c r="F13" s="5"/>
       <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="3"/>
-      <c r="J13" s="66"/>
-    </row>
-    <row r="14" spans="2:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="B14" s="65">
-        <v>12</v>
-      </c>
-      <c r="C14" s="2"/>
-      <c r="D14" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="E14" s="4"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="66"/>
+    </row>
+    <row r="14" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+      <c r="A14" s="65">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2"/>
+      <c r="C14" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="D14" s="4"/>
+      <c r="E14" s="5"/>
       <c r="F14" s="5"/>
       <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="3"/>
-      <c r="J14" s="66"/>
-    </row>
-    <row r="15" spans="2:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="B15" s="65">
-        <v>13</v>
-      </c>
-      <c r="C15" s="2"/>
-      <c r="D15" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="E15" s="4"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="66"/>
+    </row>
+    <row r="15" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+      <c r="A15" s="65">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2"/>
+      <c r="C15" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="D15" s="4"/>
+      <c r="E15" s="5"/>
       <c r="F15" s="5"/>
       <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
-      <c r="I15" s="3"/>
-      <c r="J15" s="66"/>
-    </row>
-    <row r="16" spans="2:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="B16" s="65">
-        <v>14</v>
-      </c>
-      <c r="C16" s="2"/>
-      <c r="D16" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="E16" s="4"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="66"/>
+    </row>
+    <row r="16" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+      <c r="A16" s="65">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2"/>
+      <c r="C16" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="D16" s="4"/>
+      <c r="E16" s="5"/>
       <c r="F16" s="5"/>
       <c r="G16" s="5"/>
-      <c r="H16" s="5"/>
-      <c r="I16" s="3"/>
-      <c r="J16" s="66"/>
-    </row>
-    <row r="17" spans="2:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="B17" s="65">
-        <v>15</v>
-      </c>
-      <c r="C17" s="2"/>
-      <c r="D17" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="E17" s="4"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="66"/>
+    </row>
+    <row r="17" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+      <c r="A17" s="65">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2"/>
+      <c r="C17" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="D17" s="4"/>
+      <c r="E17" s="5"/>
       <c r="F17" s="5"/>
       <c r="G17" s="5"/>
-      <c r="H17" s="5"/>
-      <c r="I17" s="3"/>
-      <c r="J17" s="66"/>
-    </row>
-    <row r="18" spans="2:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="B18" s="65">
-        <v>16</v>
-      </c>
-      <c r="C18" s="2"/>
-      <c r="D18" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="E18" s="4"/>
+      <c r="H17" s="3"/>
+      <c r="I17" s="66"/>
+    </row>
+    <row r="18" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+      <c r="A18" s="65">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2"/>
+      <c r="C18" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="D18" s="4"/>
+      <c r="E18" s="5"/>
       <c r="F18" s="5"/>
       <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
-      <c r="I18" s="3"/>
-      <c r="J18" s="66"/>
-    </row>
-    <row r="19" spans="2:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="B19" s="65">
-        <v>17</v>
-      </c>
-      <c r="C19" s="2"/>
-      <c r="D19" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="E19" s="4"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="66"/>
+    </row>
+    <row r="19" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+      <c r="A19" s="65">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2"/>
+      <c r="C19" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="D19" s="4"/>
+      <c r="E19" s="5"/>
       <c r="F19" s="5"/>
       <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
-      <c r="I19" s="3"/>
-      <c r="J19" s="66"/>
-    </row>
-    <row r="20" spans="2:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="B20" s="65">
-        <v>18</v>
-      </c>
-      <c r="C20" s="2"/>
-      <c r="D20" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="E20" s="4"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="66"/>
+    </row>
+    <row r="20" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+      <c r="A20" s="65">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2"/>
+      <c r="C20" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D20" s="4"/>
+      <c r="E20" s="5"/>
       <c r="F20" s="5"/>
       <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
-      <c r="I20" s="3"/>
-      <c r="J20" s="66"/>
-    </row>
-    <row r="21" spans="2:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="B21" s="65">
-        <v>19</v>
-      </c>
-      <c r="C21" s="2"/>
-      <c r="D21" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="E21" s="4"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="66"/>
+    </row>
+    <row r="21" spans="1:9" ht="19" x14ac:dyDescent="0.2">
+      <c r="A21" s="67">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3"/>
+      <c r="C21" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="D21" s="58"/>
+      <c r="E21" s="5"/>
       <c r="F21" s="5"/>
       <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
-      <c r="I21" s="3"/>
-      <c r="J21" s="66"/>
-    </row>
-    <row r="22" spans="2:10" ht="19" x14ac:dyDescent="0.2">
-      <c r="B22" s="67">
-        <v>20</v>
-      </c>
-      <c r="C22" s="3"/>
-      <c r="D22" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="E22" s="58"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="68"/>
+    </row>
+    <row r="22" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+      <c r="A22" s="65">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2"/>
+      <c r="C22" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="D22" s="4"/>
+      <c r="E22" s="5"/>
       <c r="F22" s="5"/>
       <c r="G22" s="5"/>
-      <c r="H22" s="5"/>
-      <c r="I22" s="3"/>
-      <c r="J22" s="68"/>
-    </row>
-    <row r="23" spans="2:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="B23" s="65">
-        <v>21</v>
-      </c>
-      <c r="C23" s="2"/>
-      <c r="D23" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="E23" s="4"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="66"/>
+    </row>
+    <row r="23" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+      <c r="A23" s="65">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2"/>
+      <c r="C23" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="D23" s="4"/>
+      <c r="E23" s="5"/>
       <c r="F23" s="5"/>
       <c r="G23" s="5"/>
-      <c r="H23" s="5"/>
-      <c r="I23" s="3"/>
-      <c r="J23" s="66"/>
-    </row>
-    <row r="24" spans="2:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="B24" s="65">
-        <v>22</v>
-      </c>
-      <c r="C24" s="2"/>
-      <c r="D24" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="E24" s="4"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="66"/>
+    </row>
+    <row r="24" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+      <c r="A24" s="65">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2"/>
+      <c r="C24" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="D24" s="4"/>
+      <c r="E24" s="5"/>
       <c r="F24" s="5"/>
       <c r="G24" s="5"/>
-      <c r="H24" s="5"/>
-      <c r="I24" s="3"/>
-      <c r="J24" s="66"/>
-    </row>
-    <row r="25" spans="2:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="B25" s="65">
-        <v>23</v>
-      </c>
-      <c r="C25" s="2"/>
-      <c r="D25" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="E25" s="4"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="66"/>
+    </row>
+    <row r="25" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+      <c r="A25" s="65">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2"/>
+      <c r="C25" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="D25" s="4"/>
+      <c r="E25" s="5"/>
       <c r="F25" s="5"/>
       <c r="G25" s="5"/>
-      <c r="H25" s="5"/>
-      <c r="I25" s="3"/>
-      <c r="J25" s="66"/>
-    </row>
-    <row r="26" spans="2:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="B26" s="65">
-        <v>24</v>
-      </c>
-      <c r="C26" s="2"/>
-      <c r="D26" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="E26" s="4"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="66"/>
+    </row>
+    <row r="26" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+      <c r="A26" s="65">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2"/>
+      <c r="C26" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="D26" s="4"/>
+      <c r="E26" s="5"/>
       <c r="F26" s="5"/>
       <c r="G26" s="5"/>
-      <c r="H26" s="5"/>
-      <c r="I26" s="3"/>
-      <c r="J26" s="66"/>
-    </row>
-    <row r="27" spans="2:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="B27" s="65">
-        <v>25</v>
-      </c>
-      <c r="C27" s="2"/>
-      <c r="D27" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="E27" s="4"/>
+      <c r="H26" s="3"/>
+      <c r="I26" s="66"/>
+    </row>
+    <row r="27" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+      <c r="A27" s="65">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2"/>
+      <c r="C27" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="D27" s="4"/>
+      <c r="E27" s="5"/>
       <c r="F27" s="5"/>
       <c r="G27" s="5"/>
-      <c r="H27" s="5"/>
-      <c r="I27" s="3"/>
-      <c r="J27" s="66"/>
-    </row>
-    <row r="28" spans="2:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="B28" s="65">
-        <v>26</v>
-      </c>
-      <c r="C28" s="2"/>
-      <c r="D28" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="E28" s="4"/>
+      <c r="H27" s="3"/>
+      <c r="I27" s="66"/>
+    </row>
+    <row r="28" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+      <c r="A28" s="65">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2"/>
+      <c r="C28" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="D28" s="4"/>
+      <c r="E28" s="5"/>
       <c r="F28" s="5"/>
       <c r="G28" s="5"/>
-      <c r="H28" s="5"/>
-      <c r="I28" s="3"/>
-      <c r="J28" s="66"/>
-    </row>
-    <row r="29" spans="2:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="B29" s="65">
-        <v>27</v>
-      </c>
-      <c r="C29" s="2"/>
-      <c r="D29" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="E29" s="4"/>
+      <c r="H28" s="3"/>
+      <c r="I28" s="66"/>
+    </row>
+    <row r="29" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+      <c r="A29" s="65">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2"/>
+      <c r="C29" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="D29" s="4"/>
+      <c r="E29" s="5"/>
       <c r="F29" s="5"/>
       <c r="G29" s="5"/>
-      <c r="H29" s="5"/>
-      <c r="I29" s="3"/>
-      <c r="J29" s="66"/>
-    </row>
-    <row r="30" spans="2:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="B30" s="65">
-        <v>28</v>
-      </c>
-      <c r="C30" s="2"/>
-      <c r="D30" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="E30" s="4"/>
+      <c r="H29" s="3"/>
+      <c r="I29" s="66"/>
+    </row>
+    <row r="30" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+      <c r="A30" s="65">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2"/>
+      <c r="C30" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="D30" s="4"/>
+      <c r="E30" s="5"/>
       <c r="F30" s="5"/>
       <c r="G30" s="5"/>
-      <c r="H30" s="5"/>
-      <c r="I30" s="3"/>
-      <c r="J30" s="66"/>
-    </row>
-    <row r="31" spans="2:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="B31" s="65">
-        <v>29</v>
-      </c>
-      <c r="C31" s="2"/>
-      <c r="D31" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="E31" s="4"/>
+      <c r="H30" s="3"/>
+      <c r="I30" s="66"/>
+    </row>
+    <row r="31" spans="1:9" ht="19" x14ac:dyDescent="0.2">
+      <c r="A31" s="67">
+        <v>30</v>
+      </c>
+      <c r="B31" s="3"/>
+      <c r="C31" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="D31" s="58"/>
+      <c r="E31" s="5"/>
       <c r="F31" s="5"/>
       <c r="G31" s="5"/>
-      <c r="H31" s="5"/>
-      <c r="I31" s="3"/>
-      <c r="J31" s="66"/>
-    </row>
-    <row r="32" spans="2:10" ht="19" x14ac:dyDescent="0.2">
-      <c r="B32" s="67">
-        <v>30</v>
-      </c>
-      <c r="C32" s="3"/>
-      <c r="D32" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="E32" s="58"/>
+      <c r="H31" s="3"/>
+      <c r="I31" s="68"/>
+    </row>
+    <row r="32" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+      <c r="A32" s="65">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2"/>
+      <c r="C32" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="D32" s="4"/>
+      <c r="E32" s="5"/>
       <c r="F32" s="5"/>
       <c r="G32" s="5"/>
-      <c r="H32" s="5"/>
-      <c r="I32" s="3"/>
-      <c r="J32" s="68"/>
-    </row>
-    <row r="33" spans="2:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="B33" s="65">
-        <v>31</v>
-      </c>
-      <c r="C33" s="2"/>
-      <c r="D33" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="E33" s="4"/>
+      <c r="H32" s="3"/>
+      <c r="I32" s="66"/>
+    </row>
+    <row r="33" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+      <c r="A33" s="65">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2"/>
+      <c r="C33" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="D33" s="4"/>
+      <c r="E33" s="5"/>
       <c r="F33" s="5"/>
       <c r="G33" s="5"/>
-      <c r="H33" s="5"/>
-      <c r="I33" s="3"/>
-      <c r="J33" s="66"/>
-    </row>
-    <row r="34" spans="2:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="B34" s="65">
-        <v>32</v>
-      </c>
-      <c r="C34" s="2"/>
-      <c r="D34" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="E34" s="4"/>
+      <c r="H33" s="3"/>
+      <c r="I33" s="66"/>
+    </row>
+    <row r="34" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+      <c r="A34" s="65">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2"/>
+      <c r="C34" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="D34" s="4"/>
+      <c r="E34" s="5"/>
       <c r="F34" s="5"/>
       <c r="G34" s="5"/>
-      <c r="H34" s="5"/>
-      <c r="I34" s="3"/>
-      <c r="J34" s="66"/>
-    </row>
-    <row r="35" spans="2:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="B35" s="65">
-        <v>33</v>
-      </c>
-      <c r="C35" s="2"/>
-      <c r="D35" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="E35" s="4"/>
+      <c r="H34" s="3"/>
+      <c r="I34" s="66"/>
+    </row>
+    <row r="35" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+      <c r="A35" s="65">
+        <v>34</v>
+      </c>
+      <c r="B35" s="2"/>
+      <c r="C35" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="D35" s="4"/>
+      <c r="E35" s="5"/>
       <c r="F35" s="5"/>
       <c r="G35" s="5"/>
-      <c r="H35" s="5"/>
-      <c r="I35" s="3"/>
-      <c r="J35" s="66"/>
-    </row>
-    <row r="36" spans="2:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="B36" s="65">
-        <v>34</v>
-      </c>
-      <c r="C36" s="2"/>
-      <c r="D36" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="E36" s="4"/>
+      <c r="H35" s="3"/>
+      <c r="I35" s="66"/>
+    </row>
+    <row r="36" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+      <c r="A36" s="65">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2"/>
+      <c r="C36" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="D36" s="4"/>
+      <c r="E36" s="5"/>
       <c r="F36" s="5"/>
       <c r="G36" s="5"/>
-      <c r="H36" s="5"/>
-      <c r="I36" s="3"/>
-      <c r="J36" s="66"/>
-    </row>
-    <row r="37" spans="2:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="B37" s="65">
-        <v>35</v>
-      </c>
-      <c r="C37" s="2"/>
-      <c r="D37" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="E37" s="4"/>
-      <c r="F37" s="5"/>
-      <c r="G37" s="5"/>
-      <c r="H37" s="5"/>
-      <c r="I37" s="3"/>
-      <c r="J37" s="66"/>
-    </row>
-    <row r="38" spans="2:10" ht="20" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="69">
+      <c r="H36" s="3"/>
+      <c r="I36" s="66"/>
+    </row>
+    <row r="37" spans="1:9" ht="20" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="69">
         <v>36</v>
       </c>
-      <c r="C38" s="70"/>
-      <c r="D38" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="E38" s="72"/>
-      <c r="F38" s="73"/>
-      <c r="G38" s="73"/>
-      <c r="H38" s="73"/>
-      <c r="I38" s="71"/>
-      <c r="J38" s="74"/>
-    </row>
-    <row r="40" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B37" s="70"/>
+      <c r="C37" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="D37" s="72"/>
+      <c r="E37" s="73"/>
+      <c r="F37" s="73"/>
+      <c r="G37" s="73"/>
+      <c r="H37" s="71"/>
+      <c r="I37" s="74"/>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
       <c r="F40" s="6" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8D9800D-40E4-824A-898A-D7075C4FF693}">
+  <dimension ref="A1:K12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:11" ht="67" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="E1" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="F1" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="G1" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="H1" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="I1" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="J1" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="K1" s="14" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+      <c r="A2" s="55">
+        <v>1</v>
+      </c>
+      <c r="B2" s="55"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+    </row>
+    <row r="3" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+      <c r="A3" s="55">
+        <v>2</v>
+      </c>
+      <c r="B3" s="55"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+    </row>
+    <row r="4" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+      <c r="A4" s="55">
+        <v>3</v>
+      </c>
+      <c r="B4" s="55"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+    </row>
+    <row r="5" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+      <c r="A5" s="55">
+        <v>4</v>
+      </c>
+      <c r="B5" s="55"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+    </row>
+    <row r="6" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+      <c r="A6" s="55">
+        <v>5</v>
+      </c>
+      <c r="B6" s="55"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3"/>
+    </row>
+    <row r="7" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+      <c r="A7" s="55">
+        <v>6</v>
+      </c>
+      <c r="B7" s="55"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
+    </row>
+    <row r="8" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+      <c r="A8" s="55">
+        <v>7</v>
+      </c>
+      <c r="B8" s="55"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+    </row>
+    <row r="9" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+      <c r="A9" s="55">
+        <v>8</v>
+      </c>
+      <c r="B9" s="55"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
+    </row>
+    <row r="10" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+      <c r="A10" s="55">
+        <v>9</v>
+      </c>
+      <c r="B10" s="55"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+    </row>
+    <row r="11" spans="1:11" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="56">
+        <v>10</v>
+      </c>
+      <c r="B11" s="56"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="18"/>
+      <c r="F11" s="18"/>
+      <c r="G11" s="18"/>
+      <c r="H11" s="16"/>
+      <c r="I11" s="16"/>
+      <c r="J11" s="16"/>
+      <c r="K11" s="16"/>
+    </row>
+    <row r="12" spans="1:11" ht="89" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="G12" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="H12" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="I12" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="J12" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="K12" s="11" t="s">
+        <v>73</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>